<commit_message>
Corrections revue adverse (round 1) : persistance, gouvernance, prix/publication, orchestration, docs
89 défauts corrigés sur 99 confirmés ; état de sécurité persisté et fail-closed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MykNGMmExNHnMWtHwWJ6jS
</commit_message>
<xml_diff>
--- a/docs/03-finance/modele_financier.xlsx
+++ b/docs/03-finance/modele_financier.xlsx
@@ -75,7 +75,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">BP : 208,79 → 209,90 implique un pas de 10 CHF et une terminaison 9,90.</t>
+          <t xml:space="preserve">BP : 208,79 → 209,90 implique un pas de 10 CHF et une terminaison 9,90. Lecture du BP seulement : le moteur applique la grille par tranches (ligne 26).</t>
         </r>
       </text>
       <mc:AlternateContent>
@@ -91,8 +91,8 @@
               <xdr:to>
                 <xdr:col>1</xdr:col>
                 <xdr:colOff>-244</xdr:colOff>
-                <xdr:row>4</xdr:row>
-                <xdr:rowOff>1</xdr:rowOff>
+                <xdr:row>6</xdr:row>
+                <xdr:rowOff>9</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -105,7 +105,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="431">
   <si>
     <t xml:space="preserve">Modèle financier — {{NOM_BOUTIQUE}} · boutique Pokémon JCC FR, ventes Suisse</t>
   </si>
@@ -1241,19 +1241,22 @@
     <t xml:space="preserve">Prix plancher arrondi au centime</t>
   </si>
   <si>
-    <t xml:space="preserve">Pas d'arrondi du prix public</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Terminaison du prix public</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prix public arrondi vers le haut</t>
+    <t xml:space="preserve">Lecture BP — pas d'arrondi du prix public</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lecture BP — terminaison du prix public</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prix public — lecture BP (pas 10 / 9,90), différente du moteur v1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concorde avec le moteur sur le cas BP seulement (coût 50 : 89,90 ici, 83,90 moteur)</t>
   </si>
   <si>
     <t xml:space="preserve">Lecture alternative « prochain X,90 » (pas de 1 CHF)</t>
   </si>
   <si>
-    <t xml:space="preserve">Ambiguïté BP/SPEC : règle d'arrondi à trancher</t>
+    <t xml:space="preserve">Lectures du BP ; règle appliquée par le moteur : ligne 26</t>
   </si>
   <si>
     <t xml:space="preserve">Valeur BP — prix plancher</t>
@@ -1263,6 +1266,12 @@
   </si>
   <si>
     <t xml:space="preserve">n.c.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prix public moteur v1 (grille rounding_tiers, prix rentable ≥ 8 CHF par commande)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pokeshop.pricing (fait foi) : config/pricing_rules.v1.yaml, avant revérification</t>
   </si>
   <si>
     <t xml:space="preserve">Contribution d'une vente unitaire à un prix donné (cas 1)</t>
@@ -11542,10 +11551,13 @@
         <f aca="false">ROUNDUP((C17-C20)/C19,0)*C19+C20</f>
         <v>209.9</v>
       </c>
+      <c r="E21" s="16" t="s">
+        <v>381</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B22" s="12" t="n">
         <f aca="false">ROUNDUP((B17-0.9)/1,0)*1+0.9</f>
@@ -11556,12 +11568,12 @@
         <v>207.9</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B23" s="55" t="n">
         <v>208.79</v>
@@ -11572,13 +11584,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B24" s="55" t="n">
         <v>209.9</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11586,7 +11598,7 @@
         <v>327</v>
       </c>
       <c r="B25" s="43" t="str">
-        <f aca="false">IF(AND(B18=B23,ROUND(B21,2)=B24),"OK — conforme BP","ÉCART")</f>
+        <f aca="false">IF(AND(B18=B23,ROUND(B21,2)=B24,ROUND(B26,2)=B24),"OK — conforme BP","ÉCART")</f>
         <v>OK — conforme BP</v>
       </c>
       <c r="C25" s="43" t="str">
@@ -11594,9 +11606,28 @@
         <v>OK — conforme BP</v>
       </c>
     </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="43" t="s">
+        <v>387</v>
+      </c>
+      <c r="B26" s="61" t="n">
+        <f aca="false">IF(ISNUMBER(B17),IF(ROUND(MAX(B17,(B7+B9+B10+B11+B12+Plancher_CHF)/(1/(1+B14)-B8)),6)&lt;10,IF(MIN(-INT(-((ROUND(MAX(B17,(B7+B9+B10+B11+B12+Plancher_CHF)/(1/(1+B14)-B8)),6))-0.5)/1)*1+0.5,-INT(-((ROUND(MAX(B17,(B7+B9+B10+B11+B12+Plancher_CHF)/(1/(1+B14)-B8)),6))-0.9)/1)*1+0.9)&lt;10,MIN(-INT(-((ROUND(MAX(B17,(B7+B9+B10+B11+B12+Plancher_CHF)/(1/(1+B14)-B8)),6))-0.5)/1)*1+0.5,-INT(-((ROUND(MAX(B17,(B7+B9+B10+B11+B12+Plancher_CHF)/(1/(1+B14)-B8)),6))-0.9)/1)*1+0.9),10.9),IF(ROUND(MAX(B17,(B7+B9+B10+B11+B12+Plancher_CHF)/(1/(1+B14)-B8)),6)&lt;100,IF(-INT(-((ROUND(MAX(B17,(B7+B9+B10+B11+B12+Plancher_CHF)/(1/(1+B14)-B8)),6))-0.9)/1)*1+0.9&lt;100,-INT(-((ROUND(MAX(B17,(B7+B9+B10+B11+B12+Plancher_CHF)/(1/(1+B14)-B8)),6))-0.9)/1)*1+0.9,104.9),MIN(-INT(-((ROUND(MAX(B17,(B7+B9+B10+B11+B12+Plancher_CHF)/(1/(1+B14)-B8)),6))-4.9)/10)*10+4.9,-INT(-((ROUND(MAX(B17,(B7+B9+B10+B11+B12+Plancher_CHF)/(1/(1+B14)-B8)),6))-9.9)/10)*10+9.9))),"n.c.")</f>
+        <v>209.9</v>
+      </c>
+      <c r="C26" s="61" t="n">
+        <f aca="false">IF(ISNUMBER(C17),IF(ROUND(MAX(C17,(C7+C9+C10+C11+C12+Plancher_CHF)/(1/(1+C14)-C8)),6)&lt;10,IF(MIN(-INT(-((ROUND(MAX(C17,(C7+C9+C10+C11+C12+Plancher_CHF)/(1/(1+C14)-C8)),6))-0.5)/1)*1+0.5,-INT(-((ROUND(MAX(C17,(C7+C9+C10+C11+C12+Plancher_CHF)/(1/(1+C14)-C8)),6))-0.9)/1)*1+0.9)&lt;10,MIN(-INT(-((ROUND(MAX(C17,(C7+C9+C10+C11+C12+Plancher_CHF)/(1/(1+C14)-C8)),6))-0.5)/1)*1+0.5,-INT(-((ROUND(MAX(C17,(C7+C9+C10+C11+C12+Plancher_CHF)/(1/(1+C14)-C8)),6))-0.9)/1)*1+0.9),10.9),IF(ROUND(MAX(C17,(C7+C9+C10+C11+C12+Plancher_CHF)/(1/(1+C14)-C8)),6)&lt;100,IF(-INT(-((ROUND(MAX(C17,(C7+C9+C10+C11+C12+Plancher_CHF)/(1/(1+C14)-C8)),6))-0.9)/1)*1+0.9&lt;100,-INT(-((ROUND(MAX(C17,(C7+C9+C10+C11+C12+Plancher_CHF)/(1/(1+C14)-C8)),6))-0.9)/1)*1+0.9,104.9),MIN(-INT(-((ROUND(MAX(C17,(C7+C9+C10+C11+C12+Plancher_CHF)/(1/(1+C14)-C8)),6))-4.9)/10)*10+4.9,-INT(-((ROUND(MAX(C17,(C7+C9+C10+C11+C12+Plancher_CHF)/(1/(1+C14)-C8)),6))-9.9)/10)*10+9.9))),"n.c.")</f>
+        <v>209.9</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>388</v>
+      </c>
+    </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -11608,27 +11639,27 @@
         <v>151</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="B29" s="11" t="n">
         <v>199.9</v>
       </c>
       <c r="C29" s="12" t="n">
-        <f aca="false">B21</f>
+        <f aca="false">B26</f>
         <v>209.9</v>
       </c>
       <c r="D29" s="55" t="n">
@@ -11637,7 +11668,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B30" s="12" t="n">
         <f aca="false">B29/(1+$B$14)</f>
@@ -11657,7 +11688,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="B31" s="12" t="n">
         <f aca="false">$B$8*B29+$B$9</f>
@@ -11677,7 +11708,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="B32" s="12" t="n">
         <f aca="false">B30-$B$7-B31-$B$10-$B$11-$B$12</f>
@@ -11697,7 +11728,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B33" s="62" t="n">
         <f aca="false">B32/B30</f>
@@ -11717,7 +11748,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="B34" s="7" t="str">
         <f aca="false">IF(B33&gt;=$B$13,"oui","NON — sous la cible")</f>
@@ -11730,7 +11761,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="B35" s="7" t="str">
         <f aca="false">IF(AND(B33&gt;=Plancher_pct,B32&gt;=Plancher_CHF),"oui","NON — blocage")</f>
@@ -11773,17 +11804,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -11809,7 +11840,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="B6" s="49" t="n">
         <f aca="false">Hypothèses!B27</f>
@@ -11829,7 +11860,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="B7" s="17" t="n">
         <f aca="false">B6*Panier_HT</f>
@@ -11869,7 +11900,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="B9" s="17" t="n">
         <f aca="false">B7*B8</f>
@@ -11889,7 +11920,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="B10" s="17" t="n">
         <f aca="false">Stock_initial</f>
@@ -11909,7 +11940,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="B11" s="51" t="n">
         <f aca="false">IF(B9&gt;0,B10/B9,0)</f>
@@ -11929,7 +11960,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="B12" s="48" t="n">
         <f aca="false">B11*Jours_mois</f>
@@ -11944,12 +11975,12 @@
         <v>7.31503759398496</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="B13" s="17" t="n">
         <f aca="false">MAX(0,B9-B10)</f>
@@ -11969,7 +12000,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="C14" s="45" t="n">
         <v>6152</v>
@@ -11981,7 +12012,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -12007,7 +12038,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">B9/Jours_mois</f>
@@ -12022,12 +12053,12 @@
         <v>410.114091890225</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="B19" s="12" t="n">
         <f aca="false">B6*Panier_TTC/Jours_mois</f>
@@ -12042,12 +12073,12 @@
         <v>633.333333333333</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="B20" s="17" t="n">
         <f aca="false">B18*(Delai_prepaiement+Jours_stock)</f>
@@ -12062,12 +12093,12 @@
         <v>18045.0200431699</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="B21" s="17" t="n">
         <f aca="false">B19*Delai_PSP</f>
@@ -12082,12 +12113,12 @@
         <v>4433.33333333333</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="B22" s="17" t="n">
         <f aca="false">B18*Credit_fournisseur</f>
@@ -12102,12 +12133,12 @@
         <v>0</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="43" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="B23" s="44" t="n">
         <f aca="false">B20+B21-B22</f>
@@ -12122,12 +12153,12 @@
         <v>22478.3533765032</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="B24" s="13" t="n">
         <f aca="false">Stock_initial+'Budget initial'!B11</f>
@@ -12142,12 +12173,12 @@
         <v>4600</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="43" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="B25" s="44" t="n">
         <f aca="false">MAX(0,B23-B24)</f>
@@ -12162,12 +12193,12 @@
         <v>17878.3533765032</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>

</xml_diff>

<commit_message>
Corrections revue adverse (round 2) : capital propriétaire, taux de change, dépublication, recette sync, règles non signées
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MykNGMmExNHnMWtHwWJ6jS
</commit_message>
<xml_diff>
--- a/docs/03-finance/modele_financier.xlsx
+++ b/docs/03-finance/modele_financier.xlsx
@@ -386,19 +386,19 @@
     <t xml:space="preserve">Étoile polaire et stop-loss du mandat — décisions de la propriétaire</t>
   </si>
   <si>
-    <t xml:space="preserve">Capital engagé de référence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lien Budget initial (BP §3) — HYPOTHÈSE : remplacer par le capital réellement engagé</t>
+    <t xml:space="preserve">Capital engagé de référence = point zéro du stop-loss global</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HYPOTHÈSE — STOP_LOSS.md §5 option A (décision C03 à J3) : apports (Budget l. 12) − lancement assumé (l. 6 à 9) − décote prudente du stock de 30 % (ratio de liquidation 0,70) = 4 200 CHF ; remplacer par le point zéro réellement posé (POST /stoploss/baseline)</t>
   </si>
   <si>
     <t xml:space="preserve">Capital_engage</t>
   </si>
   <si>
-    <t xml:space="preserve">Stop-loss global : perte cumulée maximale</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% capital</t>
+    <t xml:space="preserve">Stop-loss global : perte de valeur nette maximale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% référence</t>
   </si>
   <si>
     <t xml:space="preserve">Mandat propriétaire — gel total, réarmement par la propriétaire uniquement</t>
@@ -407,10 +407,10 @@
     <t xml:space="preserve">StopLoss_global_pct</t>
   </si>
   <si>
-    <t xml:space="preserve">Perte cumulée déclenchant le gel global</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calcul — comparée à la contribution nette cumulée</t>
+    <t xml:space="preserve">Perte déclenchant le gel global (840 CHF au BP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calcul — définition unique du moteur (pokeshop.stoploss) ; approchée ici par la contribution nette cumulée depuis le point zéro (l'ancien seuil de 1 600 CHF sur 8 000 est caduc)</t>
   </si>
   <si>
     <t xml:space="preserve">Perte_max</t>
@@ -548,10 +548,10 @@
     <t xml:space="preserve">Solde des 8 % de CA HT restant après coût produit 70 % et contribution 22 % (BP §10), moins paiement et SAV</t>
   </si>
   <si>
-    <t xml:space="preserve">Seuil du stop-loss global (contribution nette cumulée)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20 % du capital engagé ⇒ tout gelé, retour au niveau d'autonomie 1</t>
+    <t xml:space="preserve">Seuil du stop-loss global (perte ≥ 20 % de la référence du point zéro)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perte de valeur nette ≥ 20 % du capital engagé de référence (point zéro 4 200 ⇒ 840 CHF), approchée par la contribution nette cumulée ⇒ tout gelé, retour au niveau d'autonomie 1</t>
   </si>
   <si>
     <t xml:space="preserve">Suivi dans tresorerie_13_semaines.xlsx (lignes 50-51)</t>
@@ -692,7 +692,7 @@
     <t xml:space="preserve">Global</t>
   </si>
   <si>
-    <t xml:space="preserve">Perte cumulée ≥ 20 % du capital engagé</t>
+    <t xml:space="preserve">Perte de valeur nette ≥ 20 % du capital engagé de référence (point zéro)</t>
   </si>
   <si>
     <t xml:space="preserve">TOUT gelé, retour au niveau d'autonomie 1, alerte ; réarmement par la propriétaire</t>
@@ -2729,8 +2729,8 @@
         <v>93</v>
       </c>
       <c r="B44" s="13" t="n">
-        <f aca="false">'Budget initial'!B12</f>
-        <v>8000</v>
+        <f aca="false">'Budget initial'!B12-SUM('Budget initial'!B6:B9)-(1-0.7)*'Budget initial'!B5</f>
+        <v>4200</v>
       </c>
       <c r="C44" s="7" t="s">
         <v>18</v>
@@ -2765,7 +2765,7 @@
       </c>
       <c r="B46" s="17" t="n">
         <f aca="false">Capital_engage*StopLoss_global_pct</f>
-        <v>1600</v>
+        <v>840</v>
       </c>
       <c r="C46" s="7" t="s">
         <v>18</v>
@@ -3213,7 +3213,7 @@
       <c r="D13" s="18"/>
       <c r="E13" s="25" t="n">
         <f aca="false">-Perte_max</f>
-        <v>-1600</v>
+        <v>-840</v>
       </c>
       <c r="F13" s="20" t="s">
         <v>148</v>
@@ -3839,7 +3839,7 @@
       <c r="G36" s="18"/>
       <c r="H36" s="35" t="n">
         <f aca="false">-Perte_max</f>
-        <v>-1600</v>
+        <v>-840</v>
       </c>
       <c r="I36" s="35"/>
       <c r="J36" s="18" t="s">

</xml_diff>